<commit_message>
Add Pricing Structure question (P7.Q4) to client onboarding templates
Adds a new question to both the DOCX and XLSX onboarding templates asking clients to describe their pricing structure, tiers/packages, and pricing rationale. Inserted as P7.Q4 in Pillar 7 (Revenue Model and Growth Trajectory). Updates question count from 23 to 24 across both files, including the completion formula and conditional formatting in the XLSX.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/CinaTech_Client_Onboarding_Template.xlsx
+++ b/public/CinaTech_Client_Onboarding_Template.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -591,13 +591,13 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Complete all 23 questions before submitting. The score below updates automatically.</t>
+          <t>Complete all 24 questions before submitting. The score below updates automatically.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="4">
-        <f>IF(B6&lt;&gt;"",IF(LEFT(B6,1)&lt;&gt;"[",1,0),0)+IF(B7&lt;&gt;"",IF(LEFT(B7,1)&lt;&gt;"[",1,0),0)+IF(B8&lt;&gt;"",IF(LEFT(B8,1)&lt;&gt;"[",1,0),0)+IF(B11&lt;&gt;"",IF(LEFT(B11,1)&lt;&gt;"[",1,0),0)+IF(B12&lt;&gt;"",IF(LEFT(B12,1)&lt;&gt;"[",1,0),0)+IF(B13&lt;&gt;"",IF(LEFT(B13,1)&lt;&gt;"[",1,0),0)+IF(B16&lt;&gt;"",IF(LEFT(B16,1)&lt;&gt;"[",1,0),0)+IF(B17&lt;&gt;"",IF(LEFT(B17,1)&lt;&gt;"[",1,0),0)+IF(B18&lt;&gt;"",IF(LEFT(B18,1)&lt;&gt;"[",1,0),0)+IF(B21&lt;&gt;"",IF(LEFT(B21,1)&lt;&gt;"[",1,0),0)+IF(B22&lt;&gt;"",IF(LEFT(B22,1)&lt;&gt;"[",1,0),0)+IF(B25&lt;&gt;"",IF(LEFT(B25,1)&lt;&gt;"[",1,0),0)+IF(B26&lt;&gt;"",IF(LEFT(B26,1)&lt;&gt;"[",1,0),0)+IF(B29&lt;&gt;"",IF(LEFT(B29,1)&lt;&gt;"[",1,0),0)+IF(B30&lt;&gt;"",IF(LEFT(B30,1)&lt;&gt;"[",1,0),0)+IF(B31&lt;&gt;"",IF(LEFT(B31,1)&lt;&gt;"[",1,0),0)+IF(B34&lt;&gt;"",IF(LEFT(B34,1)&lt;&gt;"[",1,0),0)+IF(B35&lt;&gt;"",IF(LEFT(B35,1)&lt;&gt;"[",1,0),0)+IF(B36&lt;&gt;"",IF(LEFT(B36,1)&lt;&gt;"[",1,0),0)+IF(B39&lt;&gt;"",IF(LEFT(B39,1)&lt;&gt;"[",1,0),0)+IF(B40&lt;&gt;"",IF(LEFT(B40,1)&lt;&gt;"[",1,0),0)+IF(B43&lt;&gt;"",IF(LEFT(B43,1)&lt;&gt;"[",1,0),0)+IF(B44&lt;&gt;"",IF(LEFT(B44,1)&lt;&gt;"[",1,0),0)</f>
+        <f>IF(B6&lt;&gt;"",IF(LEFT(B6,1)&lt;&gt;"[",1,0),0)+IF(B7&lt;&gt;"",IF(LEFT(B7,1)&lt;&gt;"[",1,0),0)+IF(B8&lt;&gt;"",IF(LEFT(B8,1)&lt;&gt;"[",1,0),0)+IF(B11&lt;&gt;"",IF(LEFT(B11,1)&lt;&gt;"[",1,0),0)+IF(B12&lt;&gt;"",IF(LEFT(B12,1)&lt;&gt;"[",1,0),0)+IF(B13&lt;&gt;"",IF(LEFT(B13,1)&lt;&gt;"[",1,0),0)+IF(B16&lt;&gt;"",IF(LEFT(B16,1)&lt;&gt;"[",1,0),0)+IF(B17&lt;&gt;"",IF(LEFT(B17,1)&lt;&gt;"[",1,0),0)+IF(B18&lt;&gt;"",IF(LEFT(B18,1)&lt;&gt;"[",1,0),0)+IF(B21&lt;&gt;"",IF(LEFT(B21,1)&lt;&gt;"[",1,0),0)+IF(B22&lt;&gt;"",IF(LEFT(B22,1)&lt;&gt;"[",1,0),0)+IF(B25&lt;&gt;"",IF(LEFT(B25,1)&lt;&gt;"[",1,0),0)+IF(B26&lt;&gt;"",IF(LEFT(B26,1)&lt;&gt;"[",1,0),0)+IF(B29&lt;&gt;"",IF(LEFT(B29,1)&lt;&gt;"[",1,0),0)+IF(B30&lt;&gt;"",IF(LEFT(B30,1)&lt;&gt;"[",1,0),0)+IF(B31&lt;&gt;"",IF(LEFT(B31,1)&lt;&gt;"[",1,0),0)+IF(B34&lt;&gt;"",IF(LEFT(B34,1)&lt;&gt;"[",1,0),0)+IF(B35&lt;&gt;"",IF(LEFT(B35,1)&lt;&gt;"[",1,0),0)+IF(B36&lt;&gt;"",IF(LEFT(B36,1)&lt;&gt;"[",1,0),0)+IF(B37&lt;&gt;"",IF(LEFT(B37,1)&lt;&gt;"[",1,0),0)+IF(B40&lt;&gt;"",IF(LEFT(B40,1)&lt;&gt;"[",1,0),0)+IF(B41&lt;&gt;"",IF(LEFT(B41,1)&lt;&gt;"[",1,0),0)+IF(B44&lt;&gt;"",IF(LEFT(B44,1)&lt;&gt;"[",1,0),0)+IF(B45&lt;&gt;"",IF(LEFT(B45,1)&lt;&gt;"[",1,0),0)</f>
         <v/>
       </c>
       <c r="C3" s="5" t="n"/>
@@ -1028,125 +1028,143 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="10" customHeight="1">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="6" t="n"/>
-    </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="7" t="inlineStr">
+    <row r="37" ht="65" customHeight="1">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>P7 Q4 — Pricing Structure
+How is your service or product currently priced? Please include your pricing structure, any tiers or packages you offer, and how you arrived at these prices (e.g. cost-plus, value-based, competitor benchmarking).</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>[Pricing model / tier or package names and prices / rationale for pricing approach]</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Include specific price points or ranges if possible. Note whether prices are fixed or negotiated, and whether they differ by client type or volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="10" customHeight="1">
+      <c r="A38" s="6" t="n"/>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="6" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>PILLAR 8  —  CLIENT EDUCATION AND RETENTION</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="65" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="40" ht="65" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>P8 Q1 — Post-sign education
 What structured onboarding, training, or education do you provide to clients after they sign?</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>[Structured education / onboarding steps provided after sign-up]</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>Include kick-off calls, welcome sequences, resource libraries, portal access, check-in cadence. 'Nothing formal' is a valid answer.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="65" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="41" ht="65" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>P8 Q2 — At-risk management
 How do you identify and manage at-risk clients? What is your average client lifespan in months?</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>[At-risk signals / management process / average client lifespan in months]</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
         <is>
           <t>Name your early-warning signals: missed calls, low engagement, payment delays, complaints. Describe what action you take when you spot them.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="10" customHeight="1">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="6" t="n"/>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
+    <row r="42" ht="10" customHeight="1">
+      <c r="A42" s="6" t="n"/>
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="6" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
         <is>
           <t>PILLAR 9  —  REGULATORY AND COMPLIANCE EXPOSURE</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="65" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
+    <row r="44" ht="65" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>P9 Q1 — Sector
 What sector do you operate in? Select from the dropdown.</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>[Select your sector from the dropdown]</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
         <is>
           <t>Your sector determines which regulatory frameworks apply (CQC, MHRA, FCA, SRA, Ofsted, etc.). This is mandatory for compliance analysis.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="65" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="45" ht="65" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>P9 Q2 — Guarantees
 Do you make guarantees or promises of specific results in your marketing or contracts? Describe them exactly.</t>
         </is>
       </c>
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
         <is>
           <t>[Exact wording of any guarantees or specific result promises, or 'None']</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
+      <c r="C45" s="10" t="inlineStr">
         <is>
           <t>Copy the exact wording from your sales page, ads, or contract. Vague answers make compliance review impossible. 'We guarantee results' is not enough.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="10" customHeight="1">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="6" t="n"/>
+    <row r="46" ht="10" customHeight="1">
+      <c r="A46" s="6" t="n"/>
+      <c r="B46" s="6" t="n"/>
+      <c r="C46" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A43:C43"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:C39"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A24:C24"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:B3">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$A$3&gt;=23</formula>
+      <formula>$A$3&gt;=24</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>$A$3&gt;=18</formula>
@@ -1159,7 +1177,7 @@
     <dataValidation sqref="B29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Please select a delivery model from the list provided." promptTitle="Delivery Model" prompt="Select the model that best describes your service delivery." type="list">
       <formula1>"Done-for-you,Done-with-you,Self-serve,Hybrid,Mixed"</formula1>
     </dataValidation>
-    <dataValidation sqref="B43" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Please select your sector from the list provided." promptTitle="Sector" prompt="Select the sector that best describes your business." type="list">
+    <dataValidation sqref="B44" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Please select your sector from the list provided." promptTitle="Sector" prompt="Select the sector that best describes your business." type="list">
       <formula1>"Healthcare,Aesthetics,Financial Services,Legal,Education,Coaching/Consulting,E-commerce,SaaS/Tech,Other"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>